<commit_message>
Removing sheets for cleanliness and consistancy
</commit_message>
<xml_diff>
--- a/SPFL 2020-2021.xlsx
+++ b/SPFL 2020-2021.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JohnJ\OneDrive\Desktop\UNI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1569bcbbaf889fe0/Documents/GitHub/SPFL dissertation/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2572D4FD-534E-4581-A72E-AAEEBE461A7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -10146,6 +10146,130 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{32A2BE3E-F700-4D1A-B76E-D5CE898646E3}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
+  <location ref="A19:B32" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="11">
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0" sortType="ascending">
+      <items count="13">
+        <item x="11"/>
+        <item x="10"/>
+        <item x="8"/>
+        <item x="4"/>
+        <item x="7"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="5"/>
+        <item x="0"/>
+        <item x="6"/>
+        <item x="1"/>
+        <item x="9"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="0"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField numFmtId="1" showAll="0"/>
+    <pivotField axis="axisPage" dataField="1" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="13">
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="5" item="0" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Count of Result" fld="5" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="0" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{66FCF026-C073-4F27-84F6-A8C68093D5D5}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
   <location ref="A3:B16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="11">
@@ -10264,130 +10388,6 @@
   </dataFields>
   <chartFormats count="1">
     <chartFormat chart="0" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{32A2BE3E-F700-4D1A-B76E-D5CE898646E3}" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="1">
-  <location ref="A19:B32" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
-  <pivotFields count="11">
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0" sortType="ascending">
-      <items count="13">
-        <item x="11"/>
-        <item x="10"/>
-        <item x="8"/>
-        <item x="4"/>
-        <item x="7"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="5"/>
-        <item x="0"/>
-        <item x="6"/>
-        <item x="1"/>
-        <item x="9"/>
-        <item t="default"/>
-      </items>
-      <autoSortScope>
-        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
-          <references count="1">
-            <reference field="4294967294" count="1" selected="0">
-              <x v="0"/>
-            </reference>
-          </references>
-        </pivotArea>
-      </autoSortScope>
-    </pivotField>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField numFmtId="1" showAll="0"/>
-    <pivotField axis="axisPage" dataField="1" showAll="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="13">
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="10"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="11"/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <pageFields count="1">
-    <pageField fld="5" item="0" hier="-1"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField name="Count of Result" fld="5" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="0" format="0" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">

</xml_diff>